<commit_message>
Support IVA/total fields and update Excel writer
</commit_message>
<xml_diff>
--- a/src/assets/templates/plantilla_XML_volumetricos.xlsx
+++ b/src/assets/templates/plantilla_XML_volumetricos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documents\GitHub\XML_Volumetricos\src\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0641500B-8CF7-4118-8776-8FB3EB1797A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF14C7C-0E88-4C1B-955B-C5DEC2AE5B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{8158983C-E886-4970-9415-612054D79253}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8158983C-E886-4970-9415-612054D79253}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen_General" sheetId="1" r:id="rId1"/>
@@ -44,10 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
-  <si>
-    <t xml:space="preserve">ArchivoXML </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Serie</t>
   </si>
@@ -125,13 +122,42 @@
   </si>
   <si>
     <t>Detalle</t>
+  </si>
+  <si>
+    <t>BaseIVA</t>
+  </si>
+  <si>
+    <t>TasaIVA</t>
+  </si>
+  <si>
+    <t>IVA</t>
+  </si>
+  <si>
+    <t>Total de registros</t>
+  </si>
+  <si>
+    <t>Litros totales</t>
+  </si>
+  <si>
+    <t>Total IVA</t>
+  </si>
+  <si>
+    <t>Total facturado</t>
+  </si>
+  <si>
+    <t>Total Importe</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.0000000000_-;\-* #,##0.0000000000_-;_-* &quot;-&quot;??????????_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;* #,##0.0000_-;\-&quot;$&quot;* #,##0.0000_-;_-&quot;$&quot;* &quot;-&quot;????_-;_-@_-"/>
+  </numFmts>
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,6 +198,37 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u val="singleAccounting"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -309,41 +366,74 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,147 +768,222 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{007A9FCE-3ADA-4CF6-B04A-B642D2F2522A}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="20.88671875" customWidth="1"/>
-    <col min="4" max="4" width="16.21875" customWidth="1"/>
-    <col min="5" max="5" width="20.88671875" customWidth="1"/>
-    <col min="6" max="6" width="20.44140625" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="4" max="4" width="16.21875" style="6" customWidth="1"/>
+    <col min="5" max="5" width="20.88671875" style="9" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" style="9" customWidth="1"/>
+    <col min="7" max="7" width="15" style="9" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+    </row>
+    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="15"/>
+      <c r="E3" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="15"/>
+      <c r="G3" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="15"/>
+    </row>
+    <row r="4" spans="1:8" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="24"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="22">
+        <f>SUM(H9:H1000)</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="23"/>
+    </row>
+    <row r="5" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="15"/>
+      <c r="E5" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="15"/>
+      <c r="G5" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="15"/>
+    </row>
+    <row r="6" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="16">
+        <f>SUM(C9:C1000)</f>
+        <v>0</v>
+      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="18">
+        <f>SUM(E9:E1000)</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="19"/>
+      <c r="E6" s="20">
+        <f>SUM(F9:F1000)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="19"/>
+      <c r="G6" s="20">
+        <f>SUM(G9:G1000)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="19"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="4"/>
-    </row>
-    <row r="4" spans="1:6" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="8"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="11" t="s">
+      <c r="C8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D9" s="9"/>
+    </row>
+    <row r="11" spans="1:8" ht="16.2" x14ac:dyDescent="0.45">
+      <c r="E11" s="11"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E12" s="12"/>
+      <c r="G12" s="12"/>
+    </row>
+    <row r="14" spans="1:8" ht="16.2" x14ac:dyDescent="0.45">
+      <c r="F14" s="11"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C15" s="5"/>
+    </row>
+    <row r="18" spans="3:4" ht="16.2" x14ac:dyDescent="0.45">
+      <c r="D18" s="8"/>
+    </row>
+    <row r="23" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C23" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="17">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5B56CED-18DD-4AF9-84D8-81A7085E373B}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
     <col min="4" max="4" width="13.88671875" customWidth="1"/>
     <col min="6" max="6" width="14.33203125" customWidth="1"/>
     <col min="7" max="7" width="17.109375" customWidth="1"/>
+    <col min="9" max="10" width="11.5546875" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="11" t="s">
+      <c r="G1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="H1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -827,7 +992,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80201E91-1A02-4911-9EF9-F7D076C7B732}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" customWidth="1"/>
@@ -835,60 +1000,68 @@
     <col min="6" max="6" width="13.44140625" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="13.109375" customWidth="1"/>
-    <col min="10" max="10" width="15.6640625" customWidth="1"/>
-    <col min="11" max="11" width="16.5546875" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" style="31"/>
+    <col min="10" max="10" width="15.6640625" style="31" customWidth="1"/>
+    <col min="11" max="11" width="16.5546875" style="31" customWidth="1"/>
+    <col min="12" max="15" width="11.5546875" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="G1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="14" t="s">
+      <c r="J1" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="K1" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="D6" s="15"/>
+      <c r="L1" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" s="33" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="D6" s="5"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G20" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -909,31 +1082,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="11" t="s">
+      <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E7" s="15"/>
+      <c r="E7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -941,6 +1107,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="54aa5b16-e0f6-4b65-87da-a13075573b59" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E74234429D78DE49B21F9BD5B6CBB0EF" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5a638874e13c1008b2279be3c69f9a9c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="56198c53-886f-49c6-b799-d7dcda4c1fa6" xmlns:ns4="54aa5b16-e0f6-4b65-87da-a13075573b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a6663efd5c30af5dbe69c8e0aa6ea757" ns3:_="" ns4:_="">
     <xsd:import namespace="56198c53-886f-49c6-b799-d7dcda4c1fa6"/>
@@ -1161,7 +1335,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1170,15 +1344,24 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="54aa5b16-e0f6-4b65-87da-a13075573b59" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AC5B5C3-0232-445B-8333-805A20D5F4DA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="54aa5b16-e0f6-4b65-87da-a13075573b59"/>
+    <ds:schemaRef ds:uri="56198c53-886f-49c6-b799-d7dcda4c1fa6"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96297BDA-2061-4DE9-9202-D51E5E205D35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1197,27 +1380,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52A12B17-AC94-4DD8-B732-0C1A507189EF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AC5B5C3-0232-445B-8333-805A20D5F4DA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="54aa5b16-e0f6-4b65-87da-a13075573b59"/>
-    <ds:schemaRef ds:uri="56198c53-886f-49c6-b799-d7dcda4c1fa6"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add cfdi-transformer and validator; update docs
</commit_message>
<xml_diff>
--- a/src/assets/templates/plantilla_XML_volumetricos.xlsx
+++ b/src/assets/templates/plantilla_XML_volumetricos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documents\GitHub\XML_Volumetricos\src\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF14C7C-0E88-4C1B-955B-C5DEC2AE5B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8D8E60-553E-4F7E-A36F-F92655A13CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8158983C-E886-4970-9415-612054D79253}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
   <si>
     <t>Serie</t>
   </si>
@@ -115,15 +115,9 @@
     <t>Moneda</t>
   </si>
   <si>
-    <t>Nivel</t>
-  </si>
-  <si>
     <t>Mensaje</t>
   </si>
   <si>
-    <t>Detalle</t>
-  </si>
-  <si>
     <t>BaseIVA</t>
   </si>
   <si>
@@ -146,6 +140,36 @@
   </si>
   <si>
     <t>Total Importe</t>
+  </si>
+  <si>
+    <t>Estatus</t>
+  </si>
+  <si>
+    <t>serie</t>
+  </si>
+  <si>
+    <t>folio</t>
+  </si>
+  <si>
+    <t>fecha</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Total conceptos</t>
+  </si>
+  <si>
+    <t>Conceptos includios</t>
+  </si>
+  <si>
+    <t>ConceptosExcluidos</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Participa en Totales</t>
   </si>
 </sst>
 </file>
@@ -366,7 +390,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -380,13 +404,39 @@
     <xf numFmtId="166" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -404,36 +454,6 @@
     <xf numFmtId="166" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -782,88 +802,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
     </row>
     <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="13" t="s">
+      <c r="B3" s="16"/>
+      <c r="C3" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="14" t="s">
+      <c r="D3" s="17"/>
+      <c r="E3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="15"/>
-      <c r="G3" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="H3" s="15"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="17"/>
     </row>
     <row r="4" spans="1:8" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="24"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="22">
+      <c r="A4" s="21"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="18">
         <f>SUM(H9:H1000)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="23"/>
+      <c r="H4" s="19"/>
     </row>
     <row r="5" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="C5" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="17"/>
+      <c r="E5" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="17"/>
+      <c r="G5" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="15"/>
-      <c r="G5" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="15"/>
+      <c r="H5" s="17"/>
     </row>
     <row r="6" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="16">
+      <c r="A6" s="26">
         <f>SUM(C9:C1000)</f>
         <v>0</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="18">
+      <c r="B6" s="27"/>
+      <c r="C6" s="28">
         <f>SUM(E9:E1000)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20">
+      <c r="D6" s="29"/>
+      <c r="E6" s="30">
         <f>SUM(F9:F1000)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="19"/>
-      <c r="G6" s="20">
+      <c r="F6" s="29"/>
+      <c r="G6" s="30">
         <f>SUM(G9:G1000)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="29"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -882,7 +902,7 @@
         <v>7</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>15</v>
@@ -904,8 +924,12 @@
     <row r="14" spans="1:8" ht="16.2" x14ac:dyDescent="0.45">
       <c r="F14" s="11"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="16.2" x14ac:dyDescent="0.45">
       <c r="C15" s="5"/>
+      <c r="D15" s="8"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B16" s="5"/>
     </row>
     <row r="18" spans="3:4" ht="16.2" x14ac:dyDescent="0.45">
       <c r="D18" s="8"/>
@@ -915,6 +939,14 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:H6"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="G4:H4"/>
@@ -924,14 +956,6 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -940,17 +964,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5B56CED-18DD-4AF9-84D8-81A7085E373B}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
     <col min="4" max="4" width="13.88671875" customWidth="1"/>
     <col min="6" max="6" width="14.33203125" customWidth="1"/>
     <col min="7" max="7" width="17.109375" customWidth="1"/>
-    <col min="9" max="10" width="11.5546875" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -975,15 +998,21 @@
       <c r="H1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="29" t="s">
+      <c r="I1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="30" t="s">
+      <c r="L1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="L9" s="5"/>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -992,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80201E91-1A02-4911-9EF9-F7D076C7B732}">
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" customWidth="1"/>
@@ -1000,13 +1029,13 @@
     <col min="6" max="6" width="13.44140625" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="13.109375" customWidth="1"/>
-    <col min="9" max="9" width="11.5546875" style="31"/>
-    <col min="10" max="10" width="15.6640625" style="31" customWidth="1"/>
-    <col min="11" max="11" width="16.5546875" style="31" customWidth="1"/>
-    <col min="12" max="15" width="11.5546875" style="31"/>
+    <col min="10" max="10" width="15.6640625" customWidth="1"/>
+    <col min="11" max="11" width="16.5546875" customWidth="1"/>
+    <col min="17" max="17" width="20.33203125" customWidth="1"/>
+    <col min="18" max="18" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>11</v>
       </c>
@@ -1031,32 +1060,41 @@
       <c r="H1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="32" t="s">
+      <c r="I1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="32" t="s">
+      <c r="J1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="K1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="33" t="s">
+      <c r="L1" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="M1" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="33" t="s">
-        <v>28</v>
-      </c>
-      <c r="O1" s="33" t="s">
+      <c r="O1" s="13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="P1" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="D6" s="5"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
@@ -1071,34 +1109,55 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CB6671E-F861-4690-9D8F-F13BF7708DE9}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.77734375" customWidth="1"/>
     <col min="2" max="2" width="17.44140625" customWidth="1"/>
     <col min="3" max="3" width="13.5546875" customWidth="1"/>
-    <col min="4" max="4" width="20.88671875" customWidth="1"/>
-    <col min="5" max="5" width="47.5546875" customWidth="1"/>
+    <col min="4" max="5" width="20.88671875" customWidth="1"/>
+    <col min="6" max="6" width="23.77734375" customWidth="1"/>
+    <col min="7" max="7" width="25.77734375" customWidth="1"/>
+    <col min="8" max="8" width="11.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L1" s="5"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="E7" s="5"/>
     </row>
   </sheetData>
@@ -1115,6 +1174,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E74234429D78DE49B21F9BD5B6CBB0EF" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5a638874e13c1008b2279be3c69f9a9c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="56198c53-886f-49c6-b799-d7dcda4c1fa6" xmlns:ns4="54aa5b16-e0f6-4b65-87da-a13075573b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a6663efd5c30af5dbe69c8e0aa6ea757" ns3:_="" ns4:_="">
     <xsd:import namespace="56198c53-886f-49c6-b799-d7dcda4c1fa6"/>
@@ -1335,15 +1403,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0AC5B5C3-0232-445B-8333-805A20D5F4DA}">
   <ds:schemaRefs>
@@ -1362,6 +1421,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52A12B17-AC94-4DD8-B732-0C1A507189EF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96297BDA-2061-4DE9-9202-D51E5E205D35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1378,12 +1445,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52A12B17-AC94-4DD8-B732-0C1A507189EF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>